<commit_message>
Time Record User changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0013748_VerifyNewTitleRateSheetAvailability_CalculatedAmountOnTimeRecordManagerAfterAddingRateSheet.xlsx
+++ b/TestData/LV_TMTT0013748_VerifyNewTitleRateSheetAvailability_CalculatedAmountOnTimeRecordManagerAfterAddingRateSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598F7273-B6E5-41A3-8E9F-93538EDFECEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719B9B85-C23C-41C0-ABF5-9294EB01876E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="763" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="117">
   <si>
     <t>Rate Sheet</t>
   </si>
@@ -282,9 +282,6 @@
     <t>Roman Debald</t>
   </si>
   <si>
-    <t>Ayati Arvind</t>
-  </si>
-  <si>
     <t>Bryan Loh</t>
   </si>
   <si>
@@ -381,9 +378,6 @@
     <t>Liz Hedgcock</t>
   </si>
   <si>
-    <t>Brian Zimmerman</t>
-  </si>
-  <si>
     <t>Michael Graham</t>
   </si>
   <si>
@@ -391,6 +385,15 @@
   </si>
   <si>
     <t xml:space="preserve">Need to add on TT Beta Grp </t>
+  </si>
+  <si>
+    <t>Qi Chen</t>
+  </si>
+  <si>
+    <t>Garrett Riffe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayati Arvind </t>
   </si>
 </sst>
 </file>
@@ -1256,24 +1259,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" t="s">
         <v>84</v>
-      </c>
-      <c r="B2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C2" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1288,12 +1291,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1311,22 +1314,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1450,7 +1453,7 @@
         <v>30</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>31</v>
@@ -1470,7 +1473,7 @@
         <v>60</v>
       </c>
       <c r="D2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E2" t="s">
         <v>34</v>
@@ -1503,13 +1506,13 @@
         <v>2</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="R2" t="s">
         <v>40</v>
@@ -1518,7 +1521,7 @@
         <v>40</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U2" t="s">
         <v>41</v>
@@ -1539,13 +1542,13 @@
         <v>45</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AB2" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC2" t="s">
         <v>98</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>99</v>
       </c>
       <c r="AD2" t="s">
         <v>46</v>
@@ -1568,13 +1571,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1582,10 +1585,10 @@
         <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1641,7 +1644,7 @@
         <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
         <v>57</v>
@@ -1679,13 +1682,13 @@
         <v>62</v>
       </c>
       <c r="B1" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="D1" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1693,32 +1696,32 @@
         <v>74</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1726,21 +1729,21 @@
         <v>74</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>106</v>
-      </c>
       <c r="C6" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1748,32 +1751,32 @@
         <v>74</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1811,16 +1814,16 @@
         <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
         <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1850,7 +1853,7 @@
         <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C5" t="s">
         <v>64</v>
@@ -1875,7 +1878,7 @@
         <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
         <v>64</v>
@@ -1889,10 +1892,13 @@
         <v>71</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C8" t="s">
         <v>64</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1900,13 +1906,13 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C9" t="s">
         <v>64</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>